<commit_message>
fix a capitalization error in the cost database + fix comment in ths exmple of the multiregion moderatr booster
</commit_message>
<xml_diff>
--- a/cost/Cost_Database.xlsx
+++ b/cost/Cost_Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannbn/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A49C757-241D-224B-8625-BF8CFCE3D588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B79ED3FA-4632-4E49-813F-E19768611E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" tabRatio="877" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2251,10 +2251,10 @@
     <t>Moderator Booster Mass Graphite</t>
   </si>
   <si>
-    <t>Moderator Booster Mass Yhx</t>
-  </si>
-  <si>
     <t>Moderator Booster Mass ZrH</t>
+  </si>
+  <si>
+    <t>Moderator Booster Mass YHx</t>
   </si>
 </sst>
 </file>
@@ -2961,21 +2961,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2983,8 +2983,8 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="11" fillId="2" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3009,14 +3009,14 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3026,7 +3026,7 @@
     <cellStyle name="Normal 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
     <cellStyle name="Normal 2 5" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
-  <dxfs count="324">
+  <dxfs count="302">
     <dxf>
       <fill>
         <patternFill>
@@ -3052,6 +3052,230 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3086,7 +3310,104 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3108,6 +3429,100 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3161,20 +3576,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
@@ -3190,6 +3591,109 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3271,78 +3775,20 @@
     <dxf>
       <font>
         <b/>
+        <i/>
       </font>
-    </dxf>
-    <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
+        <patternFill patternType="gray125"/>
       </fill>
     </dxf>
     <dxf>
       <font>
         <b/>
+        <i/>
       </font>
-    </dxf>
-    <dxf>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
+        <patternFill patternType="gray0625"/>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
     </dxf>
     <dxf>
       <fill>
@@ -3371,43 +3817,12 @@
       </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
+        <i/>
       </font>
-    </dxf>
-    <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
+        <patternFill patternType="gray125"/>
       </fill>
     </dxf>
     <dxf>
@@ -3453,128 +3868,12 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
+        <i/>
       </font>
-    </dxf>
-    <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
+        <patternFill patternType="gray125"/>
       </fill>
     </dxf>
     <dxf>
@@ -3601,161 +3900,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
@@ -3771,316 +3915,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray0625"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4144,9 +3978,79 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
       <fill>
@@ -4191,9 +4095,11 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -4202,27 +4108,6 @@
       </font>
       <fill>
         <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -4243,6 +4128,83 @@
       <fill>
         <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="gray0625"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="gray125"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="gray0625"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4275,22 +4237,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFFBA"/>
@@ -4298,109 +4244,9 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
       </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray0625"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray0625"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -4429,9 +4275,63 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <b/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -4478,6 +4378,88 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
@@ -4497,9 +4479,25 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -4524,6 +4522,99 @@
       <fill>
         <patternFill>
           <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="gray0625"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
+      <fill>
+        <patternFill patternType="gray0625"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4612,11 +4703,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
@@ -4645,18 +4731,14 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
       <fill>
@@ -4680,26 +4762,10 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
       <fill>
-        <patternFill patternType="gray0625"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="gray0625"/>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -4745,149 +4811,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
       <font>
         <b/>
       </font>
@@ -4909,14 +4832,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
+          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4924,34 +4840,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4982,79 +4870,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b/>
       </font>
@@ -5072,6 +4887,39 @@
           <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFBA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
       <fill>
@@ -5114,14 +4962,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
+          <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFFBA"/>
+          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5131,6 +4979,11 @@
           <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
     </dxf>
     <dxf>
       <fill>
@@ -5152,11 +5005,6 @@
           <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -5207,6 +5055,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="6" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFFFBA"/>
         </patternFill>
       </fill>
@@ -5215,13 +5070,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5779,7 +5627,7 @@
       <c r="S3" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="141" t="s">
+      <c r="T3" s="145" t="s">
         <v>41</v>
       </c>
       <c r="U3" s="148" t="s">
@@ -6404,13 +6252,13 @@
       <c r="R11" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="S11" s="141" t="s">
+      <c r="S11" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="T11" s="141" t="s">
+      <c r="T11" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U11" s="146" t="s">
+      <c r="U11" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="49"/>
@@ -6727,13 +6575,13 @@
       <c r="R15" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S15" s="141" t="s">
+      <c r="S15" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="T15" s="141" t="s">
+      <c r="T15" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U15" s="146" t="s">
+      <c r="U15" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V15" s="49"/>
@@ -7273,13 +7121,13 @@
       <c r="R22" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S22" s="141" t="s">
+      <c r="S22" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="T22" s="141" t="s">
+      <c r="T22" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U22" s="146" t="s">
+      <c r="U22" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V22" s="49"/>
@@ -7582,13 +7430,13 @@
       <c r="R26" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S26" s="141" t="s">
+      <c r="S26" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="T26" s="141" t="s">
+      <c r="T26" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U26" s="146" t="s">
+      <c r="U26" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V26" s="49"/>
@@ -7899,13 +7747,13 @@
       <c r="R30" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S30" s="141" t="s">
+      <c r="S30" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="T30" s="141" t="s">
+      <c r="T30" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U30" s="146" t="s">
+      <c r="U30" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V30" s="49"/>
@@ -8406,13 +8254,13 @@
       <c r="R37" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S37" s="141" t="s">
+      <c r="S37" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="T37" s="141" t="s">
+      <c r="T37" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U37" s="146" t="s">
+      <c r="U37" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V37" s="49"/>
@@ -8713,13 +8561,13 @@
       <c r="R41" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="S41" s="141" t="s">
+      <c r="S41" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="T41" s="141" t="s">
+      <c r="T41" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U41" s="146" t="s">
+      <c r="U41" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V41" s="49"/>
@@ -9074,13 +8922,13 @@
       <c r="R46" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="S46" s="141" t="s">
+      <c r="S46" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="T46" s="141" t="s">
+      <c r="T46" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U46" s="146" t="s">
+      <c r="U46" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V46" s="49"/>
@@ -9525,16 +9373,16 @@
       <c r="R52" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="S52" s="141" t="s">
+      <c r="S52" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="T52" s="141" t="s">
+      <c r="T52" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U52" s="146" t="s">
+      <c r="U52" s="144" t="s">
         <v>76</v>
       </c>
-      <c r="V52" s="147" t="s">
+      <c r="V52" s="150" t="s">
         <v>162</v>
       </c>
       <c r="W52" s="77" t="s">
@@ -9881,13 +9729,13 @@
       <c r="R57" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S57" s="141" t="s">
+      <c r="S57" s="145" t="s">
         <v>105</v>
       </c>
-      <c r="T57" s="141" t="s">
+      <c r="T57" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U57" s="146" t="s">
+      <c r="U57" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V57" s="49"/>
@@ -10190,13 +10038,13 @@
       <c r="R61" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="S61" s="141" t="s">
+      <c r="S61" s="145" t="s">
         <v>74</v>
       </c>
-      <c r="T61" s="141" t="s">
+      <c r="T61" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="U61" s="146" t="s">
+      <c r="U61" s="144" t="s">
         <v>76</v>
       </c>
       <c r="V61" s="49"/>
@@ -10694,7 +10542,7 @@
       <c r="S68" s="59" t="s">
         <v>196</v>
       </c>
-      <c r="T68" s="144" t="s">
+      <c r="T68" s="146" t="s">
         <v>197</v>
       </c>
       <c r="U68" s="56"/>
@@ -11375,10 +11223,10 @@
       <c r="S76" s="59" t="s">
         <v>209</v>
       </c>
-      <c r="T76" s="144" t="s">
+      <c r="T76" s="146" t="s">
         <v>210</v>
       </c>
-      <c r="U76" s="150" t="s">
+      <c r="U76" s="147" t="s">
         <v>211</v>
       </c>
       <c r="V76" s="59" t="s">
@@ -12293,7 +12141,7 @@
       <c r="T86" s="59" t="s">
         <v>210</v>
       </c>
-      <c r="U86" s="150" t="s">
+      <c r="U86" s="147" t="s">
         <v>211</v>
       </c>
       <c r="V86" s="49"/>
@@ -13731,7 +13579,7 @@
         <v>186</v>
       </c>
       <c r="M102" s="59" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="O102" s="49" t="s">
         <v>188</v>
@@ -13816,7 +13664,7 @@
         <v>186</v>
       </c>
       <c r="M103" s="59" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="O103" s="49" t="s">
         <v>188</v>
@@ -14025,13 +13873,13 @@
       <c r="S106" s="59" t="s">
         <v>268</v>
       </c>
-      <c r="T106" s="144" t="s">
+      <c r="T106" s="146" t="s">
         <v>269</v>
       </c>
       <c r="U106" s="149" t="s">
         <v>270</v>
       </c>
-      <c r="V106" s="144"/>
+      <c r="V106" s="146"/>
       <c r="W106" s="77" t="s">
         <v>157</v>
       </c>
@@ -15316,7 +15164,7 @@
         <v>292</v>
       </c>
       <c r="U120" s="83"/>
-      <c r="V120" s="144" t="s">
+      <c r="V120" s="146" t="s">
         <v>307</v>
       </c>
       <c r="W120" s="77" t="s">
@@ -16436,10 +16284,10 @@
       <c r="R135" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="S135" s="145" t="s">
+      <c r="S135" s="141" t="s">
         <v>340</v>
       </c>
-      <c r="T135" s="145" t="s">
+      <c r="T135" s="141" t="s">
         <v>341</v>
       </c>
       <c r="U135" s="49"/>
@@ -17006,10 +16854,10 @@
       <c r="R142" s="49" t="s">
         <v>219</v>
       </c>
-      <c r="S142" s="144" t="s">
+      <c r="S142" s="146" t="s">
         <v>350</v>
       </c>
-      <c r="T142" s="144" t="s">
+      <c r="T142" s="146" t="s">
         <v>351</v>
       </c>
       <c r="U142" s="49"/>
@@ -17778,7 +17626,7 @@
       <c r="R152" s="70" t="s">
         <v>73</v>
       </c>
-      <c r="S152" s="141" t="s">
+      <c r="S152" s="145" t="s">
         <v>316</v>
       </c>
       <c r="T152" s="46"/>
@@ -19034,14 +18882,14 @@
       <c r="P170" s="49"/>
       <c r="Q170" s="66"/>
       <c r="R170" s="49"/>
-      <c r="S170" s="144" t="s">
+      <c r="S170" s="146" t="s">
         <v>399</v>
       </c>
-      <c r="T170" s="144" t="s">
+      <c r="T170" s="146" t="s">
         <v>399</v>
       </c>
       <c r="U170" s="49"/>
-      <c r="V170" s="144" t="s">
+      <c r="V170" s="146" t="s">
         <v>400</v>
       </c>
       <c r="W170" s="77"/>
@@ -19673,6 +19521,43 @@
   </sheetData>
   <autoFilter ref="A1:AB181" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="53">
+    <mergeCell ref="T26:T28"/>
+    <mergeCell ref="T41:T43"/>
+    <mergeCell ref="V106:V107"/>
+    <mergeCell ref="T61:T63"/>
+    <mergeCell ref="T76:T80"/>
+    <mergeCell ref="S135:S140"/>
+    <mergeCell ref="T11:T13"/>
+    <mergeCell ref="V170:V176"/>
+    <mergeCell ref="S30:S32"/>
+    <mergeCell ref="S15:S17"/>
+    <mergeCell ref="T37:T39"/>
+    <mergeCell ref="T46:T48"/>
+    <mergeCell ref="T22:T24"/>
+    <mergeCell ref="U52:U54"/>
+    <mergeCell ref="S26:S28"/>
+    <mergeCell ref="U26:U28"/>
+    <mergeCell ref="T52:T54"/>
+    <mergeCell ref="V120:V121"/>
+    <mergeCell ref="S152:S155"/>
+    <mergeCell ref="T142:T147"/>
+    <mergeCell ref="V52:V54"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="T57:T59"/>
+    <mergeCell ref="T15:T17"/>
+    <mergeCell ref="S41:S43"/>
+    <mergeCell ref="U106:U107"/>
+    <mergeCell ref="T68:T73"/>
+    <mergeCell ref="S46:S48"/>
+    <mergeCell ref="S22:S24"/>
+    <mergeCell ref="U22:U24"/>
+    <mergeCell ref="T30:T32"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="S11:S13"/>
+    <mergeCell ref="U11:U13"/>
+    <mergeCell ref="U37:U39"/>
+    <mergeCell ref="T106:T107"/>
     <mergeCell ref="T135:T140"/>
     <mergeCell ref="U30:U32"/>
     <mergeCell ref="S52:S54"/>
@@ -19689,331 +19574,294 @@
     <mergeCell ref="S57:S59"/>
     <mergeCell ref="S37:S39"/>
     <mergeCell ref="U86:U96"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="T57:T59"/>
-    <mergeCell ref="T15:T17"/>
-    <mergeCell ref="S41:S43"/>
-    <mergeCell ref="U106:U107"/>
-    <mergeCell ref="T68:T73"/>
-    <mergeCell ref="S46:S48"/>
-    <mergeCell ref="S22:S24"/>
-    <mergeCell ref="U22:U24"/>
-    <mergeCell ref="T30:T32"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="S11:S13"/>
-    <mergeCell ref="U11:U13"/>
-    <mergeCell ref="U37:U39"/>
-    <mergeCell ref="T106:T107"/>
-    <mergeCell ref="S135:S140"/>
-    <mergeCell ref="T11:T13"/>
-    <mergeCell ref="V170:V176"/>
-    <mergeCell ref="S30:S32"/>
-    <mergeCell ref="S15:S17"/>
-    <mergeCell ref="T37:T39"/>
-    <mergeCell ref="T46:T48"/>
-    <mergeCell ref="T22:T24"/>
-    <mergeCell ref="U52:U54"/>
-    <mergeCell ref="S26:S28"/>
-    <mergeCell ref="U26:U28"/>
-    <mergeCell ref="T52:T54"/>
-    <mergeCell ref="V120:V121"/>
-    <mergeCell ref="S152:S155"/>
-    <mergeCell ref="T142:T147"/>
-    <mergeCell ref="V52:V54"/>
-    <mergeCell ref="T26:T28"/>
-    <mergeCell ref="T41:T43"/>
-    <mergeCell ref="V106:V107"/>
-    <mergeCell ref="T61:T63"/>
-    <mergeCell ref="T76:T80"/>
   </mergeCells>
   <conditionalFormatting sqref="A97:B103">
-    <cfRule type="expression" dxfId="323" priority="572">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="322" priority="574">
+    <cfRule type="expression" dxfId="301" priority="574">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="321" priority="573">
+    <cfRule type="expression" dxfId="300" priority="573">
       <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="299" priority="572">
+      <formula>$B97=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A106:F108 U113:V119 U120:U121 A135:B140 N142:V142 N143:R143 U143:V148 K144:R144 A148:T148 T152:V157 A158:V161 A162:J163">
-    <cfRule type="expression" dxfId="320" priority="788">
+    <cfRule type="expression" dxfId="298" priority="788">
       <formula>$B106=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A97:I103">
-    <cfRule type="expression" dxfId="319" priority="35">
+    <cfRule type="expression" dxfId="297" priority="35">
       <formula>$B97=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A147:R147">
-    <cfRule type="expression" dxfId="318" priority="736">
+    <cfRule type="expression" dxfId="296" priority="736">
       <formula>$B147=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A150:R157">
-    <cfRule type="expression" dxfId="317" priority="682">
+    <cfRule type="expression" dxfId="295" priority="682">
       <formula>$B150=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="316" priority="681">
+    <cfRule type="expression" dxfId="294" priority="681">
       <formula>$B150=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="315" priority="684">
+    <cfRule type="expression" dxfId="293" priority="684">
       <formula>$B150=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="314" priority="683">
+    <cfRule type="expression" dxfId="292" priority="683">
       <formula>$B150&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A124:S125 U124:V125 U166:V168">
-    <cfRule type="expression" dxfId="313" priority="581">
+    <cfRule type="expression" dxfId="291" priority="581">
       <formula>$B124=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A105:U105">
-    <cfRule type="expression" dxfId="312" priority="792">
-      <formula>$B105=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="311" priority="790">
+    <cfRule type="expression" dxfId="290" priority="790">
       <formula>$B105=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="310" priority="789">
+    <cfRule type="expression" dxfId="289" priority="789">
       <formula>$B105=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="309" priority="791">
+    <cfRule type="expression" dxfId="288" priority="791">
       <formula>$B105&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="287" priority="792">
+      <formula>$B105=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A74:V96 A104:V104 A170:R176">
-    <cfRule type="expression" dxfId="308" priority="488">
+    <cfRule type="expression" dxfId="286" priority="488">
       <formula>$B74&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="307" priority="487">
+    <cfRule type="expression" dxfId="285" priority="486">
+      <formula>$B74=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="284" priority="487">
       <formula>$B74=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="306" priority="486">
-      <formula>$B74=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A76:V83">
-    <cfRule type="expression" dxfId="305" priority="576">
+    <cfRule type="expression" dxfId="283" priority="576">
       <formula>$B76=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A95:V96 D97:D103 A122:V123 A126:V140 A141:AG144 A145:G146 I145:AG146 A147:AG169">
-    <cfRule type="expression" dxfId="304" priority="621">
+    <cfRule type="expression" dxfId="282" priority="621">
       <formula>$B95&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A109:V111 U113:V119 U120:U121 A124:S125 U124:V125 A141:AG144 A145:G146 I145:AG146 A147:AG169 A135:B140 U135:V140 U143:V148 A5:S6 A106:F108 A1:AG4 U5:AG6">
-    <cfRule type="expression" dxfId="303" priority="785">
+    <cfRule type="expression" dxfId="281" priority="785">
       <formula>$B1=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A122:V123 A126:V140 A95:V96 D97:D103 A141:AG144 A145:G146 I145:AG146 A147:AG169">
-    <cfRule type="expression" dxfId="302" priority="620">
+    <cfRule type="expression" dxfId="280" priority="620">
       <formula>$B95=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A122:V123">
-    <cfRule type="expression" dxfId="301" priority="756">
+    <cfRule type="expression" dxfId="279" priority="756">
       <formula>$B122=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A126:V140 A122:V123">
-    <cfRule type="expression" dxfId="300" priority="619">
+    <cfRule type="expression" dxfId="278" priority="619">
       <formula>$B122=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A149:V149">
-    <cfRule type="expression" dxfId="299" priority="717">
-      <formula>$B149=3</formula>
+    <cfRule type="expression" dxfId="277" priority="720">
+      <formula>$B149=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="298" priority="718">
+    <cfRule type="expression" dxfId="276" priority="719">
+      <formula>$B149&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="275" priority="718">
       <formula>$B149=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="297" priority="720">
-      <formula>$B149=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="296" priority="719">
-      <formula>$B149&lt;2</formula>
+    <cfRule type="expression" dxfId="274" priority="717">
+      <formula>$B149=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A178:V181">
-    <cfRule type="expression" dxfId="295" priority="652">
-      <formula>$B178=0</formula>
+    <cfRule type="expression" dxfId="273" priority="651">
+      <formula>$B178&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="294" priority="649">
+    <cfRule type="expression" dxfId="272" priority="649">
       <formula>$B178=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="293" priority="650">
+    <cfRule type="expression" dxfId="271" priority="650">
       <formula>$B178=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="292" priority="651">
-      <formula>$B178&lt;2</formula>
+    <cfRule type="expression" dxfId="270" priority="652">
+      <formula>$B178=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:AG4 A5:S6 U5:AG6 A106:F108 A109:V111 U113:V119 U120:U121 A124:S125 U124:V125 A135:B140 U135:V140 A141:V141 N142:V142 N143:R143 U143:V148 K144:R144 A148:T148 T152:V157 A158:V161 A162:J163 A164:L168 U166:V168">
-    <cfRule type="expression" dxfId="291" priority="787">
+    <cfRule type="expression" dxfId="269" priority="786">
+      <formula>$B1=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="268" priority="787">
       <formula>$B1&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="290" priority="786">
-      <formula>$B1=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:AG4 A5:S6 U5:AG6 A7:AG51 A170:R176">
-    <cfRule type="expression" dxfId="289" priority="489">
+    <cfRule type="expression" dxfId="267" priority="489">
       <formula>$B1=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7:AG48">
-    <cfRule type="expression" dxfId="288" priority="551">
+    <cfRule type="expression" dxfId="266" priority="551">
       <formula>$B7=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="287" priority="552">
+    <cfRule type="expression" dxfId="265" priority="553">
+      <formula>$B7&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="264" priority="552">
       <formula>$B7=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="286" priority="553">
-      <formula>$B7&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49:AG51 F52:AG52 A52:E54 F53:U54 W53:AG54 A55:AG75 A76:V82 A83:AG84 A97:B103 A109:AG120 A121:U121 W121:AG121 A122:AG131 A132:V132 A133:Y133 A134:AG134 S170:AG170 U171:U176 W171:AG176 A177:AG181 A94:AG94">
-    <cfRule type="expression" dxfId="285" priority="750">
+    <cfRule type="expression" dxfId="263" priority="750">
       <formula>$B49=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49:AG51 F52:AG52 A52:E54 F53:U54 W53:AG54 A55:AG75 A76:V82 A83:AG84 A94:AG94 A97:B103 A109:AG120 A121:U121 W121:AG121 A122:AG131 A132:V132 A133:Y133 A134:AG134 S170:AG170 U171:U176 W171:AG176 A177:AG181">
-    <cfRule type="expression" dxfId="284" priority="751">
+    <cfRule type="expression" dxfId="262" priority="751">
       <formula>$B49&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A83:AG96">
-    <cfRule type="expression" dxfId="283" priority="64">
+    <cfRule type="expression" dxfId="261" priority="64">
       <formula>$B83=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A85:AG85">
-    <cfRule type="expression" dxfId="282" priority="61">
+    <cfRule type="expression" dxfId="260" priority="63">
+      <formula>$B85&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="259" priority="61">
       <formula>$B85=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="281" priority="62">
+    <cfRule type="expression" dxfId="258" priority="62">
       <formula>$B85=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="280" priority="63">
-      <formula>$B85&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A86:AG93">
-    <cfRule type="expression" dxfId="279" priority="522">
+    <cfRule type="expression" dxfId="257" priority="524">
+      <formula>$B86&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="256" priority="522">
       <formula>$B86=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="278" priority="523">
+    <cfRule type="expression" dxfId="255" priority="523">
       <formula>$B86=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="277" priority="524">
-      <formula>$B86&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A94:AG96 D97:D103 A145:G146 I145:R146 A147:R147">
-    <cfRule type="expression" dxfId="276" priority="733">
+    <cfRule type="expression" dxfId="254" priority="733">
       <formula>$B94=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A104:AG108">
-    <cfRule type="expression" dxfId="275" priority="506">
-      <formula>$B104=3</formula>
+    <cfRule type="expression" dxfId="253" priority="508">
+      <formula>$B104&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="274" priority="507">
+    <cfRule type="expression" dxfId="252" priority="507">
       <formula>$B104=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="273" priority="508">
-      <formula>$B104&lt;2</formula>
+    <cfRule type="expression" dxfId="251" priority="506">
+      <formula>$B104=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A133:AG134">
-    <cfRule type="expression" dxfId="272" priority="481">
+    <cfRule type="expression" dxfId="250" priority="481">
       <formula>$B133=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A141:AG144 A145:G146 I145:AG146 A147:AG169">
-    <cfRule type="expression" dxfId="271" priority="554">
+    <cfRule type="expression" dxfId="249" priority="554">
       <formula>$B141=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A177:AG181 A55:AG75 A83:AG84 A122:AG131 A132:V132 A133:Y133 A134:AG134 A109:AG120 A76:V82 A97:B103 A49:AG51 F52:AG52 F53:U54 A52:E54 W53:AG54 A121:U121 W121:AG121 S170:AG170 U171:U176 W171:AG176">
-    <cfRule type="expression" dxfId="270" priority="749">
+    <cfRule type="expression" dxfId="248" priority="749">
       <formula>$B49=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C97:C98">
-    <cfRule type="expression" dxfId="269" priority="426">
+    <cfRule type="expression" dxfId="247" priority="426">
       <formula>$B97=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="268" priority="427">
+    <cfRule type="expression" dxfId="246" priority="427">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="267" priority="428">
+    <cfRule type="expression" dxfId="245" priority="428">
       <formula>$B97&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C97:C100">
-    <cfRule type="expression" dxfId="266" priority="419">
+    <cfRule type="expression" dxfId="244" priority="419">
       <formula>$B97=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="265" priority="421">
+    <cfRule type="expression" dxfId="243" priority="420">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="242" priority="421">
       <formula>$B97&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="264" priority="420">
-      <formula>$B97=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C99:C102">
-    <cfRule type="expression" dxfId="263" priority="412">
-      <formula>$B99=3</formula>
+    <cfRule type="expression" dxfId="241" priority="414">
+      <formula>$B99&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="262" priority="413">
+    <cfRule type="expression" dxfId="240" priority="413">
       <formula>$B99=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="261" priority="414">
-      <formula>$B99&lt;2</formula>
+    <cfRule type="expression" dxfId="239" priority="412">
+      <formula>$B99=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C101:C103">
-    <cfRule type="expression" dxfId="260" priority="407">
+    <cfRule type="expression" dxfId="238" priority="405">
+      <formula>$B101=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="237" priority="407">
       <formula>$B101&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="259" priority="406">
+    <cfRule type="expression" dxfId="236" priority="406">
       <formula>$B101=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="258" priority="405">
-      <formula>$B101=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C102:C103">
-    <cfRule type="expression" dxfId="257" priority="51">
-      <formula>$B102=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="256" priority="53">
+    <cfRule type="expression" dxfId="235" priority="53">
       <formula>$B102&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="255" priority="52">
+    <cfRule type="expression" dxfId="234" priority="52">
       <formula>$B102=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="233" priority="51">
+      <formula>$B102=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C135:T135 C136:R140">
-    <cfRule type="expression" dxfId="254" priority="611">
+    <cfRule type="expression" dxfId="232" priority="609">
+      <formula>$B135=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="231" priority="611">
       <formula>$B135=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="253" priority="608">
+    <cfRule type="expression" dxfId="230" priority="610">
+      <formula>$B135&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="229" priority="608">
       <formula>$B135=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="252" priority="609">
-      <formula>$B135=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="251" priority="610">
-      <formula>$B135&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D80 D82 D84:D134 D141:D181">
@@ -20057,878 +19905,858 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D97:E103">
-    <cfRule type="expression" dxfId="250" priority="400">
+    <cfRule type="expression" dxfId="228" priority="400">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="249" priority="398">
+    <cfRule type="expression" dxfId="227" priority="399">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="226" priority="398">
       <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="248" priority="399">
-      <formula>$B97=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E97:E103">
-    <cfRule type="expression" dxfId="247" priority="397">
+    <cfRule type="expression" dxfId="225" priority="395">
+      <formula>$B97=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="224" priority="397">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="246" priority="395">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="245" priority="396">
+    <cfRule type="expression" dxfId="223" priority="396">
       <formula>$B97=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E83:Q83 Q124:Q125">
-    <cfRule type="expression" dxfId="244" priority="627">
+    <cfRule type="expression" dxfId="222" priority="627">
       <formula>_xlfn.ISFORMULA(E83)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E135:Q140">
-    <cfRule type="expression" dxfId="243" priority="607">
+    <cfRule type="expression" dxfId="221" priority="607">
       <formula>_xlfn.ISFORMULA(E135)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F102:F103 F97:I99 F100 H100:I100 F101:I101 H102:I102">
+    <cfRule type="expression" dxfId="220" priority="187">
+      <formula>$B97=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F103">
+    <cfRule type="expression" dxfId="219" priority="20">
+      <formula>$B103=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="218" priority="21">
+      <formula>$B103=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="217" priority="22">
+      <formula>$B103&lt;2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F109:F111">
-    <cfRule type="expression" dxfId="242" priority="74">
+    <cfRule type="expression" dxfId="216" priority="74">
       <formula>$B109=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F111">
-    <cfRule type="expression" dxfId="241" priority="70">
+    <cfRule type="expression" dxfId="215" priority="69">
+      <formula>$B111=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="214" priority="70">
       <formula>$B111&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="240" priority="69">
-      <formula>$B111=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="239" priority="68">
+    <cfRule type="expression" dxfId="213" priority="68">
       <formula>$B111=3</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F102:G102">
+    <cfRule type="expression" dxfId="212" priority="25">
+      <formula>$B102&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="211" priority="24">
+      <formula>$B102=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="210" priority="23">
+      <formula>$B102=3</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F109:G110">
-    <cfRule type="expression" dxfId="238" priority="73">
+    <cfRule type="expression" dxfId="209" priority="72">
+      <formula>$B109=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="208" priority="73">
       <formula>$B109&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="237" priority="72">
-      <formula>$B109=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="236" priority="71">
+    <cfRule type="expression" dxfId="207" priority="71">
       <formula>$B109=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F51:I54">
-    <cfRule type="expression" dxfId="235" priority="556">
+    <cfRule type="expression" dxfId="206" priority="556">
       <formula>$B51=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="234" priority="557">
+    <cfRule type="expression" dxfId="205" priority="557">
       <formula>$B51=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="233" priority="558">
+    <cfRule type="expression" dxfId="204" priority="559">
+      <formula>$B51=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="203" priority="558">
       <formula>$B51&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="232" priority="559">
-      <formula>$B51=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F97:I98">
-    <cfRule type="expression" dxfId="231" priority="377">
+    <cfRule type="expression" dxfId="202" priority="379">
+      <formula>$B97&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="201" priority="377">
       <formula>$B97=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="230" priority="378">
+    <cfRule type="expression" dxfId="200" priority="378">
       <formula>$B97=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="229" priority="379">
-      <formula>$B97&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F97:I99 F100 H100:I100 F101:I101 H102:I102 F102:F103">
-    <cfRule type="expression" dxfId="228" priority="189">
+    <cfRule type="expression" dxfId="199" priority="189">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="227" priority="188">
+    <cfRule type="expression" dxfId="198" priority="188">
       <formula>$B97=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="226" priority="187">
-      <formula>$B97=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F99:I101">
-    <cfRule type="expression" dxfId="225" priority="57">
-      <formula>$B99=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="224" priority="59">
+    <cfRule type="expression" dxfId="197" priority="59">
       <formula>$B99&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="223" priority="58">
+    <cfRule type="expression" dxfId="196" priority="58">
       <formula>$B99=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="195" priority="57">
+      <formula>$B99=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F102:I103">
-    <cfRule type="expression" dxfId="222" priority="34">
+    <cfRule type="expression" dxfId="194" priority="34">
       <formula>$B102&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="221" priority="33">
+    <cfRule type="expression" dxfId="193" priority="33">
       <formula>$B102=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="220" priority="32">
+    <cfRule type="expression" dxfId="192" priority="32">
       <formula>$B102=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F103:I103">
-    <cfRule type="expression" dxfId="219" priority="180">
+    <cfRule type="expression" dxfId="191" priority="181">
+      <formula>$B103=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="190" priority="180">
       <formula>$B103=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="218" priority="181">
-      <formula>$B103=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="217" priority="182">
+    <cfRule type="expression" dxfId="189" priority="182">
       <formula>$B103&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F53:U54 W53:AG54 A55:AG75 A104:AG105 A106:V109 A109:AG120 A121:U121 W121:AG121 A122:AG131 A126:V141 S170:AG170 U171:U176 W171:AG176 A177:AG181">
-    <cfRule type="expression" dxfId="216" priority="752">
+    <cfRule type="expression" dxfId="188" priority="752">
       <formula>$B53=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F52:AG52 A52:E54">
-    <cfRule type="expression" dxfId="215" priority="550">
+    <cfRule type="expression" dxfId="187" priority="550">
       <formula>$B52=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G100">
-    <cfRule type="expression" dxfId="214" priority="56">
-      <formula>$B100&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="213" priority="55">
+    <cfRule type="expression" dxfId="186" priority="55">
       <formula>$B100=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="212" priority="54">
+    <cfRule type="expression" dxfId="185" priority="54">
       <formula>$B100=3</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G102">
-    <cfRule type="expression" dxfId="211" priority="31">
-      <formula>$B102&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="210" priority="30">
-      <formula>$B102=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="209" priority="29">
-      <formula>$B102=3</formula>
+    <cfRule type="expression" dxfId="184" priority="56">
+      <formula>$B100&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G106:I107">
-    <cfRule type="expression" dxfId="208" priority="783">
+    <cfRule type="expression" dxfId="183" priority="781">
+      <formula>$B106=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="182" priority="782">
+      <formula>$B106=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="181" priority="783">
       <formula>$B106&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="207" priority="782">
-      <formula>$B106=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="206" priority="781">
-      <formula>$B106=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="205" priority="784">
+    <cfRule type="expression" dxfId="180" priority="784">
       <formula>$B106=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H145:H146 K162:L163">
-    <cfRule type="expression" dxfId="204" priority="666">
-      <formula>$B146=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="203" priority="667">
+    <cfRule type="expression" dxfId="179" priority="667">
       <formula>$B146&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="202" priority="668">
+    <cfRule type="expression" dxfId="178" priority="668">
       <formula>$B146=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="177" priority="666">
+      <formula>$B146=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H145:H146">
-    <cfRule type="expression" dxfId="201" priority="1057">
-      <formula>$B146&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="200" priority="1059">
+    <cfRule type="expression" dxfId="176" priority="1059">
       <formula>$B146=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="199" priority="1056">
+    <cfRule type="expression" dxfId="175" priority="1056">
       <formula>$B146=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="174" priority="1057">
+      <formula>$B146&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5">
-    <cfRule type="expression" dxfId="198" priority="588">
+    <cfRule type="expression" dxfId="173" priority="587">
+      <formula>$B5=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="172" priority="588">
       <formula>$B5=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="197" priority="590">
-      <formula>$B5=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="196" priority="589">
+    <cfRule type="expression" dxfId="171" priority="589">
       <formula>$B5&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="195" priority="587">
-      <formula>$B5=3</formula>
+    <cfRule type="expression" dxfId="170" priority="590">
+      <formula>$B5=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J71:L73">
-    <cfRule type="expression" dxfId="194" priority="642">
+    <cfRule type="expression" dxfId="169" priority="638">
+      <formula>_xlfn.ISFORMULA(J71)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="168" priority="642">
       <formula>$B71=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="193" priority="638">
-      <formula>_xlfn.ISFORMULA(J71)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:Q96 J104:Q1048576">
-    <cfRule type="expression" dxfId="192" priority="648">
+    <cfRule type="expression" dxfId="167" priority="648">
       <formula>_xlfn.ISFORMULA(J1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J68:Q70">
-    <cfRule type="expression" dxfId="191" priority="643">
+    <cfRule type="expression" dxfId="166" priority="643">
       <formula>_xlfn.ISFORMULA(J68)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J69:S73">
-    <cfRule type="expression" dxfId="190" priority="636">
-      <formula>$B69&lt;2</formula>
+    <cfRule type="expression" dxfId="165" priority="634">
+      <formula>$B69=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="189" priority="635">
+    <cfRule type="expression" dxfId="164" priority="635">
       <formula>$B69=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="188" priority="634">
-      <formula>$B69=3</formula>
+    <cfRule type="expression" dxfId="163" priority="636">
+      <formula>$B69&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J68:V68 J69:S70 U69:V73">
-    <cfRule type="expression" dxfId="187" priority="647">
+    <cfRule type="expression" dxfId="162" priority="647">
       <formula>$B68=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J68:V68 U69:V73">
-    <cfRule type="expression" dxfId="186" priority="646">
-      <formula>$B68&lt;2</formula>
+    <cfRule type="expression" dxfId="161" priority="644">
+      <formula>$B68=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="185" priority="645">
+    <cfRule type="expression" dxfId="160" priority="645">
       <formula>$B68=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="184" priority="644">
-      <formula>$B68=3</formula>
+    <cfRule type="expression" dxfId="159" priority="646">
+      <formula>$B68&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K81">
-    <cfRule type="expression" dxfId="183" priority="580">
+    <cfRule type="expression" dxfId="158" priority="580">
       <formula>_xlfn.ISFORMULA(K81)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K103:L103">
-    <cfRule type="expression" dxfId="182" priority="145">
-      <formula>$B103=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="181" priority="146">
-      <formula>$B103=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="180" priority="147">
-      <formula>$B103&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="K162:L163 H145:H146">
-    <cfRule type="expression" dxfId="179" priority="665">
+    <cfRule type="expression" dxfId="157" priority="665">
       <formula>$B146=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K97:M98">
-    <cfRule type="expression" dxfId="178" priority="331">
+    <cfRule type="expression" dxfId="156" priority="331">
       <formula>$B97=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="177" priority="332">
+    <cfRule type="expression" dxfId="155" priority="332">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="176" priority="333">
+    <cfRule type="expression" dxfId="154" priority="333">
       <formula>$B97&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K97:M101">
-    <cfRule type="expression" dxfId="175" priority="159">
+    <cfRule type="expression" dxfId="153" priority="159">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="174" priority="157">
+    <cfRule type="expression" dxfId="152" priority="158">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="151" priority="157">
       <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="173" priority="158">
-      <formula>$B97=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K97:M103">
-    <cfRule type="expression" dxfId="172" priority="148">
+    <cfRule type="expression" dxfId="150" priority="152">
+      <formula>$B97=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="149" priority="148">
       <formula>_xlfn.ISFORMULA(K97)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="171" priority="152">
-      <formula>$B97=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K99:M103">
-    <cfRule type="expression" dxfId="170" priority="149">
-      <formula>$B99=3</formula>
+    <cfRule type="expression" dxfId="148" priority="151">
+      <formula>$B99&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="169" priority="150">
+    <cfRule type="expression" dxfId="147" priority="150">
       <formula>$B99=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="168" priority="151">
-      <formula>$B99&lt;2</formula>
+    <cfRule type="expression" dxfId="146" priority="149">
+      <formula>$B99=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K102:M102">
-    <cfRule type="expression" dxfId="167" priority="50">
+    <cfRule type="expression" dxfId="145" priority="50">
       <formula>$B102&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="166" priority="49">
+    <cfRule type="expression" dxfId="144" priority="48">
+      <formula>$B102=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="143" priority="49">
       <formula>$B102=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="165" priority="48">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K103:M103">
+    <cfRule type="expression" dxfId="142" priority="1">
+      <formula>$B103=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="141" priority="3">
+      <formula>$B103&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="140" priority="2">
+      <formula>$B103=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K142:M143">
+    <cfRule type="expression" dxfId="139" priority="748">
+      <formula>$B142=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="138" priority="747">
+      <formula>$B142&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="137" priority="746">
+      <formula>$B142=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="136" priority="745">
+      <formula>$B142=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L112">
+    <cfRule type="expression" dxfId="135" priority="984">
+      <formula>#REF!=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="134" priority="985">
+      <formula>#REF!&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="133" priority="594">
+      <formula>$B112=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="132" priority="986">
+      <formula>#REF!=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="131" priority="987">
+      <formula>#REF!=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L112:V112">
+    <cfRule type="expression" dxfId="130" priority="593">
+      <formula>$B112&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="129" priority="591">
+      <formula>$B112=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="128" priority="592">
+      <formula>$B112=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M102:M103">
+    <cfRule type="expression" dxfId="127" priority="18">
+      <formula>$B102=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="126" priority="19">
+      <formula>$B102&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="125" priority="17">
       <formula>$B102=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K142:M143">
-    <cfRule type="expression" dxfId="164" priority="745">
-      <formula>$B142=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="163" priority="748">
-      <formula>$B142=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="162" priority="747">
-      <formula>$B142&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="161" priority="746">
-      <formula>$B142=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L112">
-    <cfRule type="expression" dxfId="160" priority="987">
-      <formula>#REF!=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="159" priority="984">
-      <formula>#REF!=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="158" priority="985">
-      <formula>#REF!&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="157" priority="594">
-      <formula>$B112=0</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="156" priority="986">
-      <formula>#REF!=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L112:V112">
-    <cfRule type="expression" dxfId="155" priority="591">
-      <formula>$B112=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="154" priority="592">
-      <formula>$B112=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="153" priority="593">
-      <formula>$B112&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="N81">
-    <cfRule type="expression" dxfId="149" priority="575">
+    <cfRule type="expression" dxfId="124" priority="575">
       <formula>_xlfn.ISFORMULA(N81)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O97:O98">
-    <cfRule type="expression" dxfId="148" priority="317">
+    <cfRule type="expression" dxfId="123" priority="316">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="122" priority="317">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="147" priority="316">
-      <formula>$B97=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="146" priority="315">
+    <cfRule type="expression" dxfId="121" priority="315">
       <formula>$B97=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O97:O103">
-    <cfRule type="expression" dxfId="145" priority="306">
+    <cfRule type="expression" dxfId="120" priority="309">
+      <formula>$B97&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="119" priority="308">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="118" priority="307">
+      <formula>$B97=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="117" priority="306">
       <formula>_xlfn.ISFORMULA(O97)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="144" priority="307">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="143" priority="308">
-      <formula>$B97=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="142" priority="309">
-      <formula>$B97&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="141" priority="310">
+    <cfRule type="expression" dxfId="116" priority="310">
       <formula>$B97=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O99:O103">
-    <cfRule type="expression" dxfId="140" priority="305">
+    <cfRule type="expression" dxfId="115" priority="305">
       <formula>$B99&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="139" priority="304">
+    <cfRule type="expression" dxfId="114" priority="303">
+      <formula>$B99=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="113" priority="304">
       <formula>$B99=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="138" priority="303">
-      <formula>$B99=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q71:Q73">
-    <cfRule type="expression" dxfId="137" priority="633">
+    <cfRule type="expression" dxfId="112" priority="633">
       <formula>_xlfn.ISFORMULA(Q71)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q97:Q103">
-    <cfRule type="expression" dxfId="136" priority="132">
+    <cfRule type="expression" dxfId="111" priority="132">
       <formula>_xlfn.ISFORMULA(Q97)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q149">
-    <cfRule type="expression" dxfId="135" priority="803">
+    <cfRule type="expression" dxfId="110" priority="802">
+      <formula>$B150=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="109" priority="803">
       <formula>$B150=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="134" priority="802">
-      <formula>$B150=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="133" priority="804">
+    <cfRule type="expression" dxfId="108" priority="804">
       <formula>$B150&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="132" priority="805">
+    <cfRule type="expression" dxfId="107" priority="805">
       <formula>$B150=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q97:R98">
-    <cfRule type="expression" dxfId="131" priority="284">
+    <cfRule type="expression" dxfId="106" priority="285">
+      <formula>$B97&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="105" priority="284">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="130" priority="283">
+    <cfRule type="expression" dxfId="104" priority="283">
       <formula>$B97=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="129" priority="285">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q97:R100">
+    <cfRule type="expression" dxfId="103" priority="276">
+      <formula>$B97=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="102" priority="277">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="101" priority="278">
       <formula>$B97&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q97:R100">
-    <cfRule type="expression" dxfId="128" priority="278">
-      <formula>$B97&lt;2</formula>
+  <conditionalFormatting sqref="Q101:R101">
+    <cfRule type="expression" dxfId="100" priority="125">
+      <formula>$B101=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="127" priority="276">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="126" priority="277">
-      <formula>$B97=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q101:R101">
-    <cfRule type="expression" dxfId="125" priority="127">
-      <formula>$B101&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="124" priority="126">
+    <cfRule type="expression" dxfId="99" priority="126">
       <formula>$B101=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="123" priority="125">
-      <formula>$B101=3</formula>
+    <cfRule type="expression" dxfId="98" priority="127">
+      <formula>$B101&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q102:R102">
-    <cfRule type="expression" dxfId="122" priority="47">
-      <formula>$B102&lt;2</formula>
+    <cfRule type="expression" dxfId="97" priority="45">
+      <formula>$B102=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="121" priority="46">
+    <cfRule type="expression" dxfId="96" priority="46">
       <formula>$B102=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="120" priority="45">
-      <formula>$B102=3</formula>
+    <cfRule type="expression" dxfId="95" priority="47">
+      <formula>$B102&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q103:R103">
-    <cfRule type="expression" dxfId="119" priority="119">
+    <cfRule type="expression" dxfId="94" priority="119">
       <formula>$B103=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="118" priority="120">
+    <cfRule type="expression" dxfId="93" priority="120">
       <formula>$B103&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="117" priority="118">
+    <cfRule type="expression" dxfId="92" priority="118">
       <formula>$B103=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q71:S73">
-    <cfRule type="expression" dxfId="116" priority="637">
+    <cfRule type="expression" dxfId="91" priority="637">
       <formula>$B71=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q99:S100">
-    <cfRule type="expression" dxfId="115" priority="269">
+    <cfRule type="expression" dxfId="90" priority="269">
       <formula>$B99=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="114" priority="270">
+    <cfRule type="expression" dxfId="89" priority="270">
       <formula>$B99=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="113" priority="271">
+    <cfRule type="expression" dxfId="88" priority="271">
       <formula>$B99&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q101:S101">
-    <cfRule type="expression" dxfId="112" priority="104">
+    <cfRule type="expression" dxfId="87" priority="106">
+      <formula>$B101&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="86" priority="104">
       <formula>$B101=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="111" priority="105">
+    <cfRule type="expression" dxfId="85" priority="105">
       <formula>$B101=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="110" priority="106">
-      <formula>$B101&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q102:S102">
-    <cfRule type="expression" dxfId="109" priority="42">
-      <formula>$B102=3</formula>
+    <cfRule type="expression" dxfId="84" priority="44">
+      <formula>$B102&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="43">
+    <cfRule type="expression" dxfId="83" priority="43">
       <formula>$B102=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="44">
-      <formula>$B102&lt;2</formula>
+    <cfRule type="expression" dxfId="82" priority="42">
+      <formula>$B102=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q103:S103">
-    <cfRule type="expression" dxfId="106" priority="113">
+    <cfRule type="expression" dxfId="81" priority="113">
       <formula>$B103&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="112">
+    <cfRule type="expression" dxfId="80" priority="111">
+      <formula>$B103=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="79" priority="112">
       <formula>$B103=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="104" priority="111">
-      <formula>$B103=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q97:T103">
-    <cfRule type="expression" dxfId="103" priority="93">
+    <cfRule type="expression" dxfId="78" priority="93">
       <formula>$B97=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S97:S100">
-    <cfRule type="expression" dxfId="102" priority="263">
+    <cfRule type="expression" dxfId="77" priority="264">
+      <formula>$B97&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="76" priority="263">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="264">
-      <formula>$B97&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="100" priority="262">
+    <cfRule type="expression" dxfId="75" priority="262">
       <formula>$B97=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S102">
-    <cfRule type="expression" dxfId="99" priority="39">
+    <cfRule type="expression" dxfId="74" priority="39">
       <formula>$B102=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="98" priority="41">
+    <cfRule type="expression" dxfId="73" priority="41">
       <formula>$B102&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="97" priority="40">
+    <cfRule type="expression" dxfId="72" priority="40">
       <formula>$B102=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S152">
-    <cfRule type="expression" dxfId="96" priority="732">
+    <cfRule type="expression" dxfId="71" priority="731">
+      <formula>$B152&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="70" priority="732">
       <formula>$B152=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="95" priority="730">
-      <formula>$B152=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="94" priority="729">
+    <cfRule type="expression" dxfId="69" priority="729">
       <formula>$B152=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="93" priority="731">
-      <formula>$B152&lt;2</formula>
+    <cfRule type="expression" dxfId="68" priority="730">
+      <formula>$B152=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S156:S157">
-    <cfRule type="expression" dxfId="92" priority="725">
+    <cfRule type="expression" dxfId="67" priority="725">
       <formula>$B156=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="91" priority="728">
+    <cfRule type="expression" dxfId="66" priority="726">
+      <formula>$B156=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="728">
       <formula>$B156=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="90" priority="727">
+    <cfRule type="expression" dxfId="64" priority="727">
       <formula>$B156&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="89" priority="726">
-      <formula>$B156=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S97:T98">
-    <cfRule type="expression" dxfId="88" priority="255">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="87" priority="256">
+    <cfRule type="expression" dxfId="63" priority="256">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="86" priority="257">
+    <cfRule type="expression" dxfId="62" priority="257">
       <formula>$B97&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="61" priority="255">
+      <formula>$B97=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S101:T101">
-    <cfRule type="expression" dxfId="85" priority="94">
-      <formula>$B101=3</formula>
+    <cfRule type="expression" dxfId="60" priority="96">
+      <formula>$B101&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="84" priority="95">
+    <cfRule type="expression" dxfId="59" priority="95">
       <formula>$B101=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="96">
-      <formula>$B101&lt;2</formula>
+    <cfRule type="expression" dxfId="58" priority="94">
+      <formula>$B101=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S103:T103">
-    <cfRule type="expression" dxfId="82" priority="90">
-      <formula>$B103=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="81" priority="92">
+    <cfRule type="expression" dxfId="57" priority="92">
       <formula>$B103&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="80" priority="91">
+    <cfRule type="expression" dxfId="56" priority="91">
       <formula>$B103=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="55" priority="90">
+      <formula>$B103=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S90:V93">
-    <cfRule type="expression" dxfId="79" priority="626">
+    <cfRule type="expression" dxfId="54" priority="626">
       <formula>$B90=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S150:V151">
-    <cfRule type="expression" dxfId="78" priority="692">
-      <formula>$B150=0</formula>
+    <cfRule type="expression" dxfId="53" priority="689">
+      <formula>$B150=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="690">
+    <cfRule type="expression" dxfId="52" priority="690">
       <formula>$B150=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="76" priority="689">
-      <formula>$B150=3</formula>
+    <cfRule type="expression" dxfId="51" priority="691">
+      <formula>$B150&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="691">
-      <formula>$B150&lt;2</formula>
+    <cfRule type="expression" dxfId="50" priority="692">
+      <formula>$B150=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5">
-    <cfRule type="expression" dxfId="74" priority="485">
+    <cfRule type="expression" dxfId="49" priority="484">
+      <formula>$B5=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="485">
       <formula>$B5&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="484">
-      <formula>$B5=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="72" priority="483">
+    <cfRule type="expression" dxfId="47" priority="483">
       <formula>$B5=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="482">
+    <cfRule type="expression" dxfId="46" priority="482">
       <formula>$B5=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T6">
-    <cfRule type="expression" dxfId="70" priority="1045">
+    <cfRule type="expression" dxfId="45" priority="1040">
+      <formula>$B5=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="1045">
       <formula>$B5=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="69" priority="1040">
-      <formula>$B5=2</formula>
+    <cfRule type="expression" dxfId="43" priority="1043">
+      <formula>$B5=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="1041">
+    <cfRule type="expression" dxfId="42" priority="1041">
       <formula>$B5&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="67" priority="1043">
-      <formula>$B5=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T97:T100">
-    <cfRule type="expression" dxfId="66" priority="248">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="65" priority="249">
+    <cfRule type="expression" dxfId="41" priority="249">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="250">
+    <cfRule type="expression" dxfId="40" priority="250">
       <formula>$B97&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="248">
+      <formula>$B97=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T99:T102">
-    <cfRule type="expression" dxfId="63" priority="97">
+    <cfRule type="expression" dxfId="38" priority="98">
+      <formula>$B99=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="37" priority="97">
       <formula>$B99=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="98">
-      <formula>$B99=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="61" priority="99">
+    <cfRule type="expression" dxfId="36" priority="99">
       <formula>$B99&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T100">
-    <cfRule type="expression" dxfId="60" priority="26">
-      <formula>$B100=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="59" priority="28">
+    <cfRule type="expression" dxfId="35" priority="28">
       <formula>$B100&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="27">
+    <cfRule type="expression" dxfId="34" priority="27">
       <formula>$B100=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="33" priority="26">
+      <formula>$B100=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T102:T103">
-    <cfRule type="expression" dxfId="57" priority="36">
-      <formula>$B102=3</formula>
+    <cfRule type="expression" dxfId="32" priority="38">
+      <formula>$B102&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="37">
+    <cfRule type="expression" dxfId="31" priority="37">
       <formula>$B102=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="38">
-      <formula>$B102&lt;2</formula>
+    <cfRule type="expression" dxfId="30" priority="36">
+      <formula>$B102=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U106">
-    <cfRule type="expression" dxfId="54" priority="813">
+    <cfRule type="expression" dxfId="29" priority="813">
       <formula>$B105=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="812">
+    <cfRule type="expression" dxfId="28" priority="812">
       <formula>$B105&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="811">
+    <cfRule type="expression" dxfId="27" priority="811">
       <formula>$B105=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="810">
+    <cfRule type="expression" dxfId="26" priority="810">
       <formula>$B105=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U135:AG140">
-    <cfRule type="expression" dxfId="50" priority="433">
+    <cfRule type="expression" dxfId="25" priority="433">
       <formula>$B135=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W97:W103">
-    <cfRule type="expression" dxfId="49" priority="239">
+    <cfRule type="expression" dxfId="24" priority="237">
+      <formula>$B97=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="238">
+      <formula>$B97=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="239">
       <formula>$B97&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="237">
-      <formula>$B97=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="47" priority="238">
-      <formula>$B97=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="46" priority="240">
+    <cfRule type="expression" dxfId="21" priority="240">
       <formula>$B97=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W76:AG82">
-    <cfRule type="expression" dxfId="45" priority="533">
+    <cfRule type="expression" dxfId="20" priority="531">
+      <formula>$B76=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="19" priority="532">
+      <formula>$B76&lt;2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="18" priority="533">
       <formula>$B76=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="532">
-      <formula>$B76&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="43" priority="531">
-      <formula>$B76=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="42" priority="530">
+    <cfRule type="expression" dxfId="17" priority="530">
       <formula>$B76=3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W95:AG96 A145:G146 I145:R146 A147:R147">
-    <cfRule type="expression" dxfId="41" priority="735">
+    <cfRule type="expression" dxfId="16" priority="734">
+      <formula>$B95=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="735">
       <formula>$B95&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="40" priority="734">
-      <formula>$B95=2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W106:AG108">
-    <cfRule type="expression" dxfId="39" priority="509">
+    <cfRule type="expression" dxfId="14" priority="509">
       <formula>$B106=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W132:AG132">
-    <cfRule type="expression" dxfId="38" priority="502">
+    <cfRule type="expression" dxfId="13" priority="503">
+      <formula>$B132=2</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="505">
+      <formula>$B132=0</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="502">
       <formula>$B132=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="503">
-      <formula>$B132=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="36" priority="504">
+    <cfRule type="expression" dxfId="10" priority="504">
       <formula>$B132&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="35" priority="505">
-      <formula>$B132=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W135:AG140">
-    <cfRule type="expression" dxfId="34" priority="430">
+    <cfRule type="expression" dxfId="9" priority="430">
       <formula>$B135=3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="431">
+    <cfRule type="expression" dxfId="8" priority="431">
       <formula>$B135=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="432">
+    <cfRule type="expression" dxfId="7" priority="432">
       <formula>$B135&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z97:AG103">
-    <cfRule type="expression" dxfId="31" priority="82">
+    <cfRule type="expression" dxfId="6" priority="82">
       <formula>$B97=0</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="81">
-      <formula>$B97&lt;2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="29" priority="80">
+    <cfRule type="expression" dxfId="5" priority="80">
       <formula>$B97=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="79">
+    <cfRule type="expression" dxfId="4" priority="79">
       <formula>$B97=3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="81">
+      <formula>$B97&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z133:AG133">
-    <cfRule type="expression" dxfId="27" priority="478">
-      <formula>$B133=3</formula>
+    <cfRule type="expression" dxfId="2" priority="480">
+      <formula>$B133&lt;2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="479">
+    <cfRule type="expression" dxfId="1" priority="479">
       <formula>$B133=2</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="480">
-      <formula>$B133&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F102">
-    <cfRule type="expression" dxfId="24" priority="23">
-      <formula>$B102=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="24">
-      <formula>$B102=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="23" priority="25">
-      <formula>$B102&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F103">
-    <cfRule type="expression" dxfId="21" priority="20">
-      <formula>$B103=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="21">
-      <formula>$B103=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="20" priority="22">
-      <formula>$B103&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M102:M103">
-    <cfRule type="expression" dxfId="17" priority="17">
-      <formula>$B102=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="18">
-      <formula>$B102=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="19">
-      <formula>$B102&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M103">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>$B103=3</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$B103=2</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>$B103&lt;2</formula>
+    <cfRule type="expression" dxfId="0" priority="478">
+      <formula>$B133=3</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="15">
@@ -24299,7 +24127,7 @@
       <c r="T3" s="160" t="s">
         <v>41</v>
       </c>
-      <c r="U3" s="163" t="s">
+      <c r="U3" s="164" t="s">
         <v>42</v>
       </c>
       <c r="V3" s="108"/>
@@ -24495,7 +24323,7 @@
       <c r="T5" s="160" t="s">
         <v>63</v>
       </c>
-      <c r="U5" s="163" t="s">
+      <c r="U5" s="164" t="s">
         <v>58</v>
       </c>
       <c r="V5" s="108"/>
@@ -24945,7 +24773,7 @@
       <c r="T11" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U11" s="162" t="s">
+      <c r="U11" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V11" s="108"/>
@@ -25498,7 +25326,7 @@
       <c r="T18" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U18" s="162" t="s">
+      <c r="U18" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V18" s="108"/>
@@ -25909,7 +25737,7 @@
       <c r="T23" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U23" s="162" t="s">
+      <c r="U23" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V23" s="108"/>
@@ -26320,7 +26148,7 @@
       <c r="T28" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U28" s="162" t="s">
+      <c r="U28" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V28" s="108"/>
@@ -26731,7 +26559,7 @@
       <c r="T33" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U33" s="162" t="s">
+      <c r="U33" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V33" s="108"/>
@@ -27142,7 +26970,7 @@
       <c r="T38" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U38" s="162" t="s">
+      <c r="U38" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V38" s="108"/>
@@ -27692,7 +27520,7 @@
       <c r="T45" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U45" s="162" t="s">
+      <c r="U45" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V45" s="108"/>
@@ -28250,7 +28078,7 @@
       <c r="T52" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U52" s="162" t="s">
+      <c r="U52" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V52" s="108"/>
@@ -28666,7 +28494,7 @@
       <c r="T57" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U57" s="162" t="s">
+      <c r="U57" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V57" s="108"/>
@@ -29084,7 +28912,7 @@
       <c r="T62" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U62" s="162" t="s">
+      <c r="U62" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V62" s="108"/>
@@ -29495,7 +29323,7 @@
       <c r="T67" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U67" s="162" t="s">
+      <c r="U67" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V67" s="108"/>
@@ -30045,7 +29873,7 @@
       <c r="T74" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U74" s="162" t="s">
+      <c r="U74" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V74" s="108"/>
@@ -30456,7 +30284,7 @@
       <c r="T79" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U79" s="162" t="s">
+      <c r="U79" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V79" s="108"/>
@@ -31019,7 +30847,7 @@
       <c r="T86" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U86" s="162" t="s">
+      <c r="U86" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V86" s="108"/>
@@ -31578,7 +31406,7 @@
       <c r="T93" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U93" s="162" t="s">
+      <c r="U93" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V93" s="108"/>
@@ -31989,7 +31817,7 @@
       <c r="T98" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U98" s="162" t="s">
+      <c r="U98" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V98" s="108"/>
@@ -32560,7 +32388,7 @@
       <c r="T105" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U105" s="162" t="s">
+      <c r="U105" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V105" s="108"/>
@@ -33131,7 +32959,7 @@
       <c r="T112" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U112" s="162" t="s">
+      <c r="U112" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V112" s="108"/>
@@ -33555,7 +33383,7 @@
       <c r="T117" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U117" s="162" t="s">
+      <c r="U117" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V117" s="108"/>
@@ -33994,7 +33822,7 @@
       <c r="T122" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U122" s="162" t="s">
+      <c r="U122" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V122" s="108"/>
@@ -34405,7 +34233,7 @@
       <c r="T127" s="160" t="s">
         <v>75</v>
       </c>
-      <c r="U127" s="162" t="s">
+      <c r="U127" s="163" t="s">
         <v>76</v>
       </c>
       <c r="V127" s="108"/>
@@ -41822,10 +41650,10 @@
       <c r="R225" s="108" t="s">
         <v>86</v>
       </c>
-      <c r="S225" s="164" t="s">
+      <c r="S225" s="162" t="s">
         <v>340</v>
       </c>
-      <c r="T225" s="164" t="s">
+      <c r="T225" s="162" t="s">
         <v>341</v>
       </c>
       <c r="U225" s="108"/>
@@ -44594,21 +44422,45 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="S23:S25"/>
-    <mergeCell ref="S225:S230"/>
-    <mergeCell ref="S122:S124"/>
-    <mergeCell ref="U57:U59"/>
-    <mergeCell ref="S38:S40"/>
-    <mergeCell ref="U62:U64"/>
-    <mergeCell ref="T117:T119"/>
-    <mergeCell ref="S112:S114"/>
-    <mergeCell ref="S57:S59"/>
-    <mergeCell ref="S28:S30"/>
-    <mergeCell ref="U28:U30"/>
-    <mergeCell ref="U93:U95"/>
-    <mergeCell ref="S127:S129"/>
-    <mergeCell ref="T225:T230"/>
-    <mergeCell ref="S74:S76"/>
+    <mergeCell ref="S242:S245"/>
+    <mergeCell ref="U33:U35"/>
+    <mergeCell ref="U98:U100"/>
+    <mergeCell ref="U67:U69"/>
+    <mergeCell ref="U117:U119"/>
+    <mergeCell ref="U52:U54"/>
+    <mergeCell ref="U79:U81"/>
+    <mergeCell ref="U38:U40"/>
+    <mergeCell ref="U112:U114"/>
+    <mergeCell ref="T122:T124"/>
+    <mergeCell ref="S67:S69"/>
+    <mergeCell ref="T67:T69"/>
+    <mergeCell ref="T127:T129"/>
+    <mergeCell ref="S18:S20"/>
+    <mergeCell ref="U122:U124"/>
+    <mergeCell ref="U18:U20"/>
+    <mergeCell ref="T79:T81"/>
+    <mergeCell ref="U127:U129"/>
+    <mergeCell ref="U23:U25"/>
+    <mergeCell ref="T105:T107"/>
+    <mergeCell ref="T52:T54"/>
+    <mergeCell ref="T86:T88"/>
+    <mergeCell ref="S93:S95"/>
+    <mergeCell ref="S62:S64"/>
+    <mergeCell ref="S33:S35"/>
+    <mergeCell ref="T23:T25"/>
+    <mergeCell ref="T28:T30"/>
+    <mergeCell ref="S45:S47"/>
+    <mergeCell ref="S79:S81"/>
+    <mergeCell ref="U3:U4"/>
+    <mergeCell ref="T57:T59"/>
+    <mergeCell ref="T33:T35"/>
+    <mergeCell ref="T18:T20"/>
+    <mergeCell ref="T98:T100"/>
+    <mergeCell ref="T45:T47"/>
+    <mergeCell ref="U5:U6"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="T5:T6"/>
+    <mergeCell ref="T11:T13"/>
     <mergeCell ref="S11:S13"/>
     <mergeCell ref="T74:T76"/>
     <mergeCell ref="T112:T114"/>
@@ -44625,45 +44477,21 @@
     <mergeCell ref="S52:S54"/>
     <mergeCell ref="S86:S88"/>
     <mergeCell ref="U86:U88"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="T57:T59"/>
-    <mergeCell ref="T33:T35"/>
-    <mergeCell ref="T18:T20"/>
-    <mergeCell ref="T98:T100"/>
-    <mergeCell ref="T45:T47"/>
-    <mergeCell ref="U5:U6"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="T5:T6"/>
-    <mergeCell ref="T11:T13"/>
-    <mergeCell ref="S18:S20"/>
-    <mergeCell ref="U122:U124"/>
-    <mergeCell ref="U18:U20"/>
-    <mergeCell ref="T79:T81"/>
-    <mergeCell ref="U127:U129"/>
-    <mergeCell ref="U23:U25"/>
-    <mergeCell ref="T105:T107"/>
-    <mergeCell ref="T52:T54"/>
-    <mergeCell ref="T86:T88"/>
-    <mergeCell ref="S93:S95"/>
-    <mergeCell ref="S62:S64"/>
-    <mergeCell ref="S33:S35"/>
-    <mergeCell ref="T23:T25"/>
-    <mergeCell ref="T28:T30"/>
-    <mergeCell ref="S45:S47"/>
-    <mergeCell ref="S79:S81"/>
-    <mergeCell ref="S242:S245"/>
-    <mergeCell ref="U33:U35"/>
-    <mergeCell ref="U98:U100"/>
-    <mergeCell ref="U67:U69"/>
-    <mergeCell ref="U117:U119"/>
-    <mergeCell ref="U52:U54"/>
-    <mergeCell ref="U79:U81"/>
-    <mergeCell ref="U38:U40"/>
-    <mergeCell ref="U112:U114"/>
-    <mergeCell ref="T122:T124"/>
-    <mergeCell ref="S67:S69"/>
-    <mergeCell ref="T67:T69"/>
-    <mergeCell ref="T127:T129"/>
+    <mergeCell ref="S23:S25"/>
+    <mergeCell ref="S225:S230"/>
+    <mergeCell ref="S122:S124"/>
+    <mergeCell ref="U57:U59"/>
+    <mergeCell ref="S38:S40"/>
+    <mergeCell ref="U62:U64"/>
+    <mergeCell ref="T117:T119"/>
+    <mergeCell ref="S112:S114"/>
+    <mergeCell ref="S57:S59"/>
+    <mergeCell ref="S28:S30"/>
+    <mergeCell ref="U28:U30"/>
+    <mergeCell ref="U93:U95"/>
+    <mergeCell ref="S127:S129"/>
+    <mergeCell ref="T225:T230"/>
+    <mergeCell ref="S74:S76"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>